<commit_message>
Update Framework Description + Add Copyright
</commit_message>
<xml_diff>
--- a/tools/excel/3cf/3cf-v3.1.xlsx
+++ b/tools/excel/3cf/3cf-v3.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\tarkadia\projects\intuitem\ciso-assistant-community\tools\excel\3cf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8A8943F-4008-4C20-9B5A-5D10D7B8DAD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5082DE17-F175-4A80-A233-CB407190951B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31680" yWindow="-11052" windowWidth="22812" windowHeight="14988" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1485" yWindow="-15870" windowWidth="25440" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1772" uniqueCount="688">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1774" uniqueCount="690">
   <si>
     <t>type</t>
   </si>
@@ -2105,11 +2105,18 @@
 Durée d’archivage : Au moins 5 ans après la création du document</t>
   </si>
   <si>
-    <t>Ce document, établi par la direction de la sécurité de l’aviation civile (DSAC) et l’OSAC, présente le Cadre de Conformité Cyber France (3CF) pour l’aviation civile.
+    <t>implementation_groups_definition</t>
+  </si>
+  <si>
+    <t>copyright</t>
+  </si>
+  <si>
+    <t>Ce document peut être utilisé librement au sein de la communauté du transport aérien et sous réserve de mentionner sa paternité (source
+et date de la dernière mise à jour).</t>
+  </si>
+  <si>
+    <t>Ce document, établi par la direction de la sécurité de l’aviation civile (DSAC) et l’organisme pour la sécurité de l’aviation civile (OSAC), présente le Cadre de Conformité Cyber France (3CF) pour l’aviation civile.
 Version 3.1 du 11 mars 2026</t>
-  </si>
-  <si>
-    <t>implementation_groups_definition</t>
   </si>
 </sst>
 </file>
@@ -2452,11 +2459,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="121.44140625" customWidth="1"/>
+    <col min="1" max="1" width="12.109375" customWidth="1"/>
+    <col min="2" max="2" width="126.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -2512,22 +2519,30 @@
         <v>12</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>686</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" t="s">
-        <v>14</v>
+        <v>687</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>688</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>15</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B10" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2541,7 +2556,7 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="111.88671875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2590,12 +2605,12 @@
         <v>12</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>686</v>
+        <v>689</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="B7" t="s">
         <v>680</v>

</xml_diff>